<commit_message>
xlsx update (remove temporary files)
</commit_message>
<xml_diff>
--- a/Data/Glados/glados.xlsx
+++ b/Data/Glados/glados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\makinoyuuki\Desktop\SANER2026\Data\Glados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\makinoyuuki\Desktop\SANER2027\Data\Glados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C61374-3899-49B9-8016-E407B0239157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1B2B93-F91C-4DA0-B7E2-FB03965E34CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{76F834DE-5EFC-4D6B-9741-493A547AC4EA}"/>
   </bookViews>

</xml_diff>